<commit_message>
Ajustes no painel: sinalizador de cor PA vs PD e formato de data DD/MM/YYYY
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcel.mfpm\Downloads\REFORMULAÇÃO - LARISSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcel.mfpm\Downloads\REFORMULAÇÃO - LARISSA\PROJETO PA E PD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF38328F-5DCB-4324-8225-CBD6D3C19A07}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C19513-3C2A-47E0-B08F-C4D1684F113D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14385" windowHeight="4065" xr2:uid="{A872491A-373F-4F8D-9252-91ADE5CA8578}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14385" windowHeight="4065" activeTab="3" xr2:uid="{A872491A-373F-4F8D-9252-91ADE5CA8578}"/>
   </bookViews>
   <sheets>
     <sheet name="EPF" sheetId="1" r:id="rId1"/>
@@ -389,6 +389,30 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -396,30 +420,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -825,7 +825,7 @@
       </c>
     </row>
     <row r="2" spans="1:16">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="32" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -857,7 +857,7 @@
       <c r="P2" s="5"/>
     </row>
     <row r="3" spans="1:16">
-      <c r="A3" s="34"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
@@ -887,7 +887,7 @@
       <c r="P3" s="4"/>
     </row>
     <row r="4" spans="1:16">
-      <c r="A4" s="34"/>
+      <c r="A4" s="32"/>
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
@@ -907,16 +907,16 @@
       <c r="H4" s="5">
         <v>15</v>
       </c>
-      <c r="I4" s="38">
-        <v>8</v>
-      </c>
-      <c r="J4" s="38">
+      <c r="I4" s="31">
+        <v>8</v>
+      </c>
+      <c r="J4" s="31">
         <v>5</v>
       </c>
       <c r="K4" s="5">
         <v>15</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="31">
         <v>10</v>
       </c>
       <c r="M4" s="6">
@@ -927,7 +927,7 @@
       <c r="P4" s="5"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="34"/>
+      <c r="A5" s="32"/>
       <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
@@ -950,13 +950,13 @@
       <c r="I5" s="5">
         <v>12</v>
       </c>
-      <c r="J5" s="38">
+      <c r="J5" s="31">
         <v>1</v>
       </c>
       <c r="K5" s="5">
         <v>17</v>
       </c>
-      <c r="L5" s="38">
+      <c r="L5" s="31">
         <v>15</v>
       </c>
       <c r="M5" s="6">
@@ -967,7 +967,7 @@
       <c r="P5" s="5"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="34"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
@@ -993,10 +993,10 @@
       <c r="J6" s="5">
         <v>8</v>
       </c>
-      <c r="K6" s="38">
+      <c r="K6" s="31">
         <v>16</v>
       </c>
-      <c r="L6" s="38">
+      <c r="L6" s="31">
         <v>8</v>
       </c>
       <c r="M6" s="6">
@@ -1007,7 +1007,7 @@
       <c r="P6" s="8"/>
     </row>
     <row r="7" spans="1:16">
-      <c r="A7" s="34"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1037,7 +1037,7 @@
       <c r="P7" s="9"/>
     </row>
     <row r="8" spans="1:16">
-      <c r="A8" s="34"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
@@ -1067,7 +1067,7 @@
       <c r="P8" s="5"/>
     </row>
     <row r="9" spans="1:16">
-      <c r="A9" s="34"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1097,7 +1097,7 @@
       <c r="P9" s="5"/>
     </row>
     <row r="10" spans="1:16">
-      <c r="A10" s="34"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
@@ -1127,7 +1127,7 @@
       <c r="P10" s="5"/>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="34"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="3" t="s">
         <v>12</v>
       </c>
@@ -1157,7 +1157,7 @@
       <c r="P11" s="10"/>
     </row>
     <row r="12" spans="1:16">
-      <c r="A12" s="34"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
@@ -1187,7 +1187,7 @@
       <c r="P12" s="5"/>
     </row>
     <row r="13" spans="1:16">
-      <c r="A13" s="34"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
@@ -1217,7 +1217,7 @@
       <c r="P13" s="5"/>
     </row>
     <row r="14" spans="1:16">
-      <c r="A14" s="34"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="3" t="s">
         <v>12</v>
       </c>
@@ -1247,7 +1247,7 @@
       <c r="P14" s="5"/>
     </row>
     <row r="15" spans="1:16">
-      <c r="A15" s="34"/>
+      <c r="A15" s="32"/>
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -1277,7 +1277,7 @@
       <c r="P15" s="5"/>
     </row>
     <row r="16" spans="1:16">
-      <c r="A16" s="34"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="3" t="s">
         <v>12</v>
       </c>
@@ -1307,7 +1307,7 @@
       <c r="P16" s="5"/>
     </row>
     <row r="17" spans="1:16">
-      <c r="A17" s="34"/>
+      <c r="A17" s="32"/>
       <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
@@ -1337,7 +1337,7 @@
       <c r="P17" s="5"/>
     </row>
     <row r="18" spans="1:16">
-      <c r="A18" s="34"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1367,7 +1367,7 @@
       <c r="P18" s="5"/>
     </row>
     <row r="19" spans="1:16">
-      <c r="A19" s="34"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
@@ -1408,8 +1408,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD951558-3DEF-4573-8D77-A22E116C5C48}">
-  <dimension ref="A1:P35"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.875" style="1"/>
     <col min="2" max="2" width="8.875" style="2"/>
@@ -1477,7 +1477,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="33" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -1509,7 +1509,7 @@
       <c r="P2" s="13"/>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1">
-      <c r="A3" s="40"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="11" t="s">
         <v>9</v>
       </c>
@@ -1539,7 +1539,7 @@
       <c r="P3" s="12"/>
     </row>
     <row r="4" spans="1:16" ht="15" customHeight="1">
-      <c r="A4" s="40"/>
+      <c r="A4" s="34"/>
       <c r="B4" s="11" t="s">
         <v>11</v>
       </c>
@@ -1562,13 +1562,13 @@
       <c r="I4" s="13">
         <v>12</v>
       </c>
-      <c r="J4" s="38">
+      <c r="J4" s="31">
         <v>1</v>
       </c>
       <c r="K4" s="13">
         <v>17</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="31">
         <v>15</v>
       </c>
       <c r="M4" s="14">
@@ -1579,7 +1579,7 @@
       <c r="P4" s="13"/>
     </row>
     <row r="5" spans="1:16" ht="15" customHeight="1">
-      <c r="A5" s="40"/>
+      <c r="A5" s="34"/>
       <c r="B5" s="11" t="s">
         <v>11</v>
       </c>
@@ -1619,7 +1619,7 @@
       <c r="P5" s="13"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1">
-      <c r="A6" s="40"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="11" t="s">
         <v>11</v>
       </c>
@@ -1645,10 +1645,10 @@
       <c r="J6" s="13">
         <v>8</v>
       </c>
-      <c r="K6" s="38">
+      <c r="K6" s="31">
         <v>16</v>
       </c>
-      <c r="L6" s="38">
+      <c r="L6" s="31">
         <v>18</v>
       </c>
       <c r="M6" s="14">
@@ -1659,7 +1659,7 @@
       <c r="P6" s="16"/>
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1">
-      <c r="A7" s="40"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="11" t="s">
         <v>11</v>
       </c>
@@ -1679,16 +1679,16 @@
       <c r="H7" s="13">
         <v>18</v>
       </c>
-      <c r="I7" s="38">
-        <v>8</v>
-      </c>
-      <c r="J7" s="38">
+      <c r="I7" s="31">
+        <v>8</v>
+      </c>
+      <c r="J7" s="31">
         <v>10</v>
       </c>
       <c r="K7" s="13">
         <v>10</v>
       </c>
-      <c r="L7" s="38">
+      <c r="L7" s="31">
         <v>16</v>
       </c>
       <c r="M7" s="13"/>
@@ -1697,7 +1697,7 @@
       <c r="P7" s="17"/>
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1">
-      <c r="A8" s="40"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="11" t="s">
         <v>11</v>
       </c>
@@ -1717,7 +1717,7 @@
       <c r="H8" s="13">
         <v>0</v>
       </c>
-      <c r="I8" s="38">
+      <c r="I8" s="31">
         <v>5</v>
       </c>
       <c r="J8" s="13">
@@ -1737,7 +1737,7 @@
       <c r="P8" s="13"/>
     </row>
     <row r="9" spans="1:16" ht="15" customHeight="1">
-      <c r="A9" s="40"/>
+      <c r="A9" s="34"/>
       <c r="B9" s="11" t="s">
         <v>11</v>
       </c>
@@ -1766,7 +1766,7 @@
       <c r="K9" s="13">
         <v>24</v>
       </c>
-      <c r="L9" s="38">
+      <c r="L9" s="31">
         <v>21</v>
       </c>
       <c r="M9" s="14">
@@ -1777,7 +1777,7 @@
       <c r="P9" s="13"/>
     </row>
     <row r="10" spans="1:16" ht="15" customHeight="1">
-      <c r="A10" s="40"/>
+      <c r="A10" s="34"/>
       <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
@@ -1797,10 +1797,10 @@
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="38">
-        <v>11</v>
-      </c>
-      <c r="J10" s="38">
+      <c r="I10" s="31">
+        <v>11</v>
+      </c>
+      <c r="J10" s="31">
         <v>0</v>
       </c>
       <c r="K10" s="13">
@@ -1817,7 +1817,7 @@
       <c r="P10" s="13"/>
     </row>
     <row r="11" spans="1:16" ht="15" customHeight="1">
-      <c r="A11" s="40"/>
+      <c r="A11" s="34"/>
       <c r="B11" s="11" t="s">
         <v>12</v>
       </c>
@@ -1847,7 +1847,7 @@
       <c r="P11" s="18"/>
     </row>
     <row r="12" spans="1:16" ht="15" customHeight="1">
-      <c r="A12" s="40"/>
+      <c r="A12" s="34"/>
       <c r="B12" s="11" t="s">
         <v>12</v>
       </c>
@@ -1877,7 +1877,7 @@
       <c r="P12" s="13"/>
     </row>
     <row r="13" spans="1:16" ht="15" customHeight="1">
-      <c r="A13" s="40"/>
+      <c r="A13" s="34"/>
       <c r="B13" s="11" t="s">
         <v>12</v>
       </c>
@@ -1907,7 +1907,7 @@
       <c r="P13" s="13"/>
     </row>
     <row r="14" spans="1:16" ht="15" customHeight="1">
-      <c r="A14" s="40"/>
+      <c r="A14" s="34"/>
       <c r="B14" s="11" t="s">
         <v>12</v>
       </c>
@@ -1937,7 +1937,7 @@
       <c r="P14" s="13"/>
     </row>
     <row r="15" spans="1:16" ht="15" customHeight="1">
-      <c r="A15" s="40"/>
+      <c r="A15" s="34"/>
       <c r="B15" s="11" t="s">
         <v>12</v>
       </c>
@@ -1967,7 +1967,7 @@
       <c r="P15" s="13"/>
     </row>
     <row r="16" spans="1:16" ht="15" customHeight="1">
-      <c r="A16" s="40"/>
+      <c r="A16" s="34"/>
       <c r="B16" s="11" t="s">
         <v>12</v>
       </c>
@@ -1997,7 +1997,7 @@
       <c r="P16" s="13"/>
     </row>
     <row r="17" spans="1:16" ht="15" customHeight="1">
-      <c r="A17" s="40"/>
+      <c r="A17" s="34"/>
       <c r="B17" s="11" t="s">
         <v>12</v>
       </c>
@@ -2027,7 +2027,7 @@
       <c r="P17" s="13"/>
     </row>
     <row r="18" spans="1:16" ht="15" customHeight="1">
-      <c r="A18" s="40"/>
+      <c r="A18" s="34"/>
       <c r="B18" s="11" t="s">
         <v>12</v>
       </c>
@@ -2057,7 +2057,7 @@
       <c r="P18" s="13"/>
     </row>
     <row r="19" spans="1:16" ht="15" customHeight="1">
-      <c r="A19" s="40"/>
+      <c r="A19" s="34"/>
       <c r="B19" s="11" t="s">
         <v>12</v>
       </c>
@@ -2086,8 +2086,8 @@
       <c r="O19" s="14"/>
       <c r="P19" s="13"/>
     </row>
-    <row r="20" spans="1:16" ht="15">
-      <c r="A20" s="40"/>
+    <row r="20" spans="1:16">
+      <c r="A20" s="34"/>
       <c r="B20" s="11" t="s">
         <v>12</v>
       </c>
@@ -2116,8 +2116,8 @@
       <c r="O20" s="13"/>
       <c r="P20" s="13"/>
     </row>
-    <row r="21" spans="1:16" ht="15">
-      <c r="A21" s="41"/>
+    <row r="21" spans="1:16">
+      <c r="A21" s="35"/>
       <c r="B21" s="11" t="s">
         <v>12</v>
       </c>
@@ -2146,20 +2146,6 @@
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
     </row>
-    <row r="22" spans="1:16" ht="15"/>
-    <row r="23" spans="1:16" ht="15"/>
-    <row r="24" spans="1:16" ht="15"/>
-    <row r="25" spans="1:16" ht="15"/>
-    <row r="26" spans="1:16" ht="15"/>
-    <row r="27" spans="1:16" ht="15"/>
-    <row r="28" spans="1:16" ht="15"/>
-    <row r="29" spans="1:16" ht="15"/>
-    <row r="30" spans="1:16" ht="15"/>
-    <row r="31" spans="1:16" ht="15"/>
-    <row r="32" spans="1:16" ht="15"/>
-    <row r="33" ht="15"/>
-    <row r="34" ht="15"/>
-    <row r="35" ht="15"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:A21"/>
@@ -2170,8 +2156,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65613A53-C102-4256-AEC9-305787A9B0EA}">
-  <dimension ref="A1:P55"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.875" style="1"/>
     <col min="2" max="2" width="8.875" style="2"/>
@@ -2239,7 +2225,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="19" t="s">
@@ -2271,7 +2257,7 @@
       <c r="P2" s="21"/>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1">
-      <c r="A3" s="36"/>
+      <c r="A3" s="37"/>
       <c r="B3" s="19" t="s">
         <v>11</v>
       </c>
@@ -2291,16 +2277,16 @@
       <c r="H3" s="21">
         <v>15</v>
       </c>
-      <c r="I3" s="38">
-        <v>8</v>
-      </c>
-      <c r="J3" s="38">
+      <c r="I3" s="31">
+        <v>8</v>
+      </c>
+      <c r="J3" s="31">
         <v>5</v>
       </c>
-      <c r="K3" s="38">
+      <c r="K3" s="31">
         <v>15</v>
       </c>
-      <c r="L3" s="38">
+      <c r="L3" s="31">
         <v>10</v>
       </c>
       <c r="M3" s="22">
@@ -2311,7 +2297,7 @@
       <c r="P3" s="21"/>
     </row>
     <row r="4" spans="1:16" ht="15" customHeight="1">
-      <c r="A4" s="36"/>
+      <c r="A4" s="37"/>
       <c r="B4" s="19" t="s">
         <v>11</v>
       </c>
@@ -2331,16 +2317,16 @@
       <c r="H4" s="21">
         <v>18</v>
       </c>
-      <c r="I4" s="38">
+      <c r="I4" s="31">
         <v>12</v>
       </c>
-      <c r="J4" s="38">
+      <c r="J4" s="31">
         <v>1</v>
       </c>
-      <c r="K4" s="38">
+      <c r="K4" s="31">
         <v>17</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="31">
         <v>15</v>
       </c>
       <c r="M4" s="22">
@@ -2351,7 +2337,7 @@
       <c r="P4" s="21"/>
     </row>
     <row r="5" spans="1:16" ht="15" customHeight="1">
-      <c r="A5" s="36"/>
+      <c r="A5" s="37"/>
       <c r="B5" s="19" t="s">
         <v>11</v>
       </c>
@@ -2381,7 +2367,7 @@
       <c r="P5" s="21"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1">
-      <c r="A6" s="37"/>
+      <c r="A6" s="38"/>
       <c r="B6" s="19" t="s">
         <v>11</v>
       </c>
@@ -2410,55 +2396,6 @@
       <c r="O6" s="22"/>
       <c r="P6" s="21"/>
     </row>
-    <row r="7" spans="1:16" ht="15"/>
-    <row r="8" spans="1:16" ht="15"/>
-    <row r="9" spans="1:16" ht="15"/>
-    <row r="10" spans="1:16" ht="15"/>
-    <row r="11" spans="1:16" ht="15"/>
-    <row r="12" spans="1:16" ht="15"/>
-    <row r="13" spans="1:16" ht="15"/>
-    <row r="14" spans="1:16" ht="15"/>
-    <row r="15" spans="1:16" ht="15"/>
-    <row r="16" spans="1:16" ht="15"/>
-    <row r="17" ht="15"/>
-    <row r="18" ht="15"/>
-    <row r="19" ht="15"/>
-    <row r="20" ht="15"/>
-    <row r="21" ht="15"/>
-    <row r="22" ht="15"/>
-    <row r="23" ht="15"/>
-    <row r="24" ht="15"/>
-    <row r="25" ht="15"/>
-    <row r="26" ht="15"/>
-    <row r="27" ht="15"/>
-    <row r="28" ht="15"/>
-    <row r="29" ht="15"/>
-    <row r="30" ht="15"/>
-    <row r="31" ht="15"/>
-    <row r="32" ht="15"/>
-    <row r="33" ht="15"/>
-    <row r="34" ht="15"/>
-    <row r="35" ht="15"/>
-    <row r="36" ht="15"/>
-    <row r="37" ht="15"/>
-    <row r="38" ht="15"/>
-    <row r="39" ht="15"/>
-    <row r="40" ht="15"/>
-    <row r="41" ht="15"/>
-    <row r="42" ht="15"/>
-    <row r="43" ht="15"/>
-    <row r="44" ht="15"/>
-    <row r="45" ht="15"/>
-    <row r="46" ht="15"/>
-    <row r="47" ht="15"/>
-    <row r="48" ht="15"/>
-    <row r="49" ht="15"/>
-    <row r="50" ht="15"/>
-    <row r="51" ht="15"/>
-    <row r="52" ht="15"/>
-    <row r="53" ht="15"/>
-    <row r="54" ht="15"/>
-    <row r="55" ht="15"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:A6"/>
@@ -2469,8 +2406,8 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF0F1BD-DA81-409F-B879-31CA2FD3E4BB}">
-  <dimension ref="A1:P55"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.875" style="1"/>
     <col min="2" max="2" width="8.875" style="2"/>
@@ -2538,7 +2475,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="39" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="24" t="s">
@@ -2570,7 +2507,7 @@
       <c r="P2" s="25"/>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1">
-      <c r="A3" s="32"/>
+      <c r="A3" s="40"/>
       <c r="B3" s="24" t="s">
         <v>11</v>
       </c>
@@ -2590,16 +2527,16 @@
       <c r="H3" s="26">
         <v>15</v>
       </c>
-      <c r="I3" s="38">
-        <v>8</v>
-      </c>
-      <c r="J3" s="38">
+      <c r="I3" s="31">
+        <v>8</v>
+      </c>
+      <c r="J3" s="31">
         <v>5</v>
       </c>
-      <c r="K3" s="38">
+      <c r="K3" s="31">
         <v>15</v>
       </c>
-      <c r="L3" s="38">
+      <c r="L3" s="31">
         <v>10</v>
       </c>
       <c r="M3" s="27">
@@ -2610,7 +2547,7 @@
       <c r="P3" s="26"/>
     </row>
     <row r="4" spans="1:16" ht="15" customHeight="1">
-      <c r="A4" s="32"/>
+      <c r="A4" s="40"/>
       <c r="B4" s="24" t="s">
         <v>11</v>
       </c>
@@ -2630,16 +2567,16 @@
       <c r="H4" s="26">
         <v>18</v>
       </c>
-      <c r="I4" s="38">
+      <c r="I4" s="31">
         <v>12</v>
       </c>
-      <c r="J4" s="38">
+      <c r="J4" s="31">
         <v>1</v>
       </c>
-      <c r="K4" s="38">
+      <c r="K4" s="31">
         <v>17</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="31">
         <v>15</v>
       </c>
       <c r="M4" s="27">
@@ -2650,7 +2587,7 @@
       <c r="P4" s="26"/>
     </row>
     <row r="5" spans="1:16" ht="15" customHeight="1">
-      <c r="A5" s="32"/>
+      <c r="A5" s="40"/>
       <c r="B5" s="24" t="s">
         <v>11</v>
       </c>
@@ -2680,7 +2617,7 @@
       <c r="P5" s="26"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1">
-      <c r="A6" s="33"/>
+      <c r="A6" s="41"/>
       <c r="B6" s="24" t="s">
         <v>11</v>
       </c>
@@ -2709,55 +2646,6 @@
       <c r="O6" s="27"/>
       <c r="P6" s="26"/>
     </row>
-    <row r="7" spans="1:16" ht="15"/>
-    <row r="8" spans="1:16" ht="15"/>
-    <row r="9" spans="1:16" ht="15"/>
-    <row r="10" spans="1:16" ht="15"/>
-    <row r="11" spans="1:16" ht="15"/>
-    <row r="12" spans="1:16" ht="15"/>
-    <row r="13" spans="1:16" ht="15"/>
-    <row r="14" spans="1:16" ht="15"/>
-    <row r="15" spans="1:16" ht="15"/>
-    <row r="16" spans="1:16" ht="15"/>
-    <row r="17" ht="15"/>
-    <row r="18" ht="15"/>
-    <row r="19" ht="15"/>
-    <row r="20" ht="15"/>
-    <row r="21" ht="15"/>
-    <row r="22" ht="15"/>
-    <row r="23" ht="15"/>
-    <row r="24" ht="15"/>
-    <row r="25" ht="15"/>
-    <row r="26" ht="15"/>
-    <row r="27" ht="15"/>
-    <row r="28" ht="15"/>
-    <row r="29" ht="15"/>
-    <row r="30" ht="15"/>
-    <row r="31" ht="15"/>
-    <row r="32" ht="15"/>
-    <row r="33" ht="15"/>
-    <row r="34" ht="15"/>
-    <row r="35" ht="15"/>
-    <row r="36" ht="15"/>
-    <row r="37" ht="15"/>
-    <row r="38" ht="15"/>
-    <row r="39" ht="15"/>
-    <row r="40" ht="15"/>
-    <row r="41" ht="15"/>
-    <row r="42" ht="15"/>
-    <row r="43" ht="15"/>
-    <row r="44" ht="15"/>
-    <row r="45" ht="15"/>
-    <row r="46" ht="15"/>
-    <row r="47" ht="15"/>
-    <row r="48" ht="15"/>
-    <row r="49" ht="15"/>
-    <row r="50" ht="15"/>
-    <row r="51" ht="15"/>
-    <row r="52" ht="15"/>
-    <row r="53" ht="15"/>
-    <row r="54" ht="15"/>
-    <row r="55" ht="15"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:A6"/>
@@ -2767,12 +2655,13 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22554d0a-1932-447e-b007-a2186b2152bd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2960,19 +2849,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22554d0a-1932-447e-b007-a2186b2152bd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D86BB587-35FF-4C72-A3B4-30D223CD8217}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D844D4EE-45BA-4D0C-B92D-0FE188981EFA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="22554d0a-1932-447e-b007-a2186b2152bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2996,17 +2892,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D844D4EE-45BA-4D0C-B92D-0FE188981EFA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D86BB587-35FF-4C72-A3B4-30D223CD8217}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="22554d0a-1932-447e-b007-a2186b2152bd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Remove preview (7).html e atualiza planilha xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcel.mfpm\Downloads\REFORMULAÇÃO - LARISSA\PROJETO PA E PD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C19513-3C2A-47E0-B08F-C4D1684F113D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8EC48C-8DFF-4EC9-9C3F-501FD289C23B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14385" windowHeight="4065" activeTab="3" xr2:uid="{A872491A-373F-4F8D-9252-91ADE5CA8578}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14390" windowHeight="4070" xr2:uid="{A872491A-373F-4F8D-9252-91ADE5CA8578}"/>
   </bookViews>
   <sheets>
     <sheet name="EPF" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="29">
   <si>
     <t>MOD.</t>
   </si>
@@ -109,12 +109,6 @@
   </si>
   <si>
     <t>VIATURA PA</t>
-  </si>
-  <si>
-    <t>24 / onibus</t>
-  </si>
-  <si>
-    <t>24/ONIBUS</t>
   </si>
   <si>
     <t>1S</t>
@@ -757,26 +751,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DF0423F-3F79-4C1A-8E98-72864AA85B9D}">
   <dimension ref="A1:P19"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.875" style="1"/>
-    <col min="2" max="2" width="8.875" style="2"/>
-    <col min="3" max="3" width="8.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="8.83203125" style="2"/>
+    <col min="3" max="3" width="8.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.58203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.58203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.08203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.25" style="1" customWidth="1"/>
-    <col min="11" max="12" width="10.625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="17.125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="10.58203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.08203125" style="1" customWidth="1"/>
     <col min="14" max="15" width="17" style="1" customWidth="1"/>
     <col min="16" max="16" width="38.5" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.875" style="1"/>
+    <col min="17" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30">
+    <row r="1" spans="1:16" ht="28">
       <c r="A1" s="5"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -926,7 +920,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" ht="14.5">
       <c r="A5" s="32"/>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -1177,11 +1171,21 @@
       <c r="H12" s="5">
         <v>0</v>
       </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="I12" s="5">
+        <v>2</v>
+      </c>
+      <c r="J12" s="5">
+        <v>4</v>
+      </c>
+      <c r="K12" s="5">
+        <v>0</v>
+      </c>
+      <c r="L12" s="5">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6">
+        <v>45798</v>
+      </c>
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
       <c r="P12" s="5"/>
@@ -1204,14 +1208,24 @@
       <c r="G13" s="5">
         <v>4</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="H13" s="5">
+        <v>24</v>
+      </c>
+      <c r="I13" s="5">
+        <v>16</v>
+      </c>
+      <c r="J13" s="5">
+        <v>14</v>
+      </c>
+      <c r="K13" s="5">
+        <v>4</v>
+      </c>
+      <c r="L13" s="31">
+        <v>20</v>
+      </c>
+      <c r="M13" s="6">
+        <v>45798</v>
+      </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
       <c r="P13" s="5"/>
@@ -1409,26 +1423,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD951558-3DEF-4573-8D77-A22E116C5C48}">
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.875" style="1"/>
-    <col min="2" max="2" width="8.875" style="2"/>
-    <col min="3" max="3" width="8.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="8.83203125" style="2"/>
+    <col min="3" max="3" width="8.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.58203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.08203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.25" style="1" customWidth="1"/>
-    <col min="11" max="12" width="10.625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="17.125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="10.58203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.08203125" style="1" customWidth="1"/>
     <col min="14" max="15" width="17" style="1" customWidth="1"/>
     <col min="16" max="16" width="38.5" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.875" style="1"/>
+    <col min="17" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30">
+    <row r="1" spans="1:16" ht="28">
       <c r="A1" s="13"/>
       <c r="B1" s="11" t="s">
         <v>0</v>
@@ -1443,7 +1457,7 @@
         <v>18</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G1" s="11" t="s">
         <v>20</v>
@@ -1867,11 +1881,21 @@
       <c r="H12" s="13">
         <v>0</v>
       </c>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
+      <c r="I12" s="13">
+        <v>2</v>
+      </c>
+      <c r="J12" s="13">
+        <v>4</v>
+      </c>
+      <c r="K12" s="13">
+        <v>0</v>
+      </c>
+      <c r="L12" s="13">
+        <v>0</v>
+      </c>
+      <c r="M12" s="14">
+        <v>45798</v>
+      </c>
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
       <c r="P12" s="13"/>
@@ -1894,14 +1918,24 @@
       <c r="G13" s="13">
         <v>4</v>
       </c>
-      <c r="H13" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
+      <c r="H13" s="13">
+        <v>24</v>
+      </c>
+      <c r="I13" s="13">
+        <v>16</v>
+      </c>
+      <c r="J13" s="13">
+        <v>14</v>
+      </c>
+      <c r="K13" s="13">
+        <v>4</v>
+      </c>
+      <c r="L13" s="31">
+        <v>20</v>
+      </c>
+      <c r="M13" s="14">
+        <v>45798</v>
+      </c>
       <c r="N13" s="14"/>
       <c r="O13" s="14"/>
       <c r="P13" s="13"/>
@@ -2017,11 +2051,21 @@
       <c r="H17" s="13">
         <v>0</v>
       </c>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
+      <c r="I17" s="31">
+        <v>5</v>
+      </c>
+      <c r="J17" s="13">
+        <v>0</v>
+      </c>
+      <c r="K17" s="13">
+        <v>0</v>
+      </c>
+      <c r="L17" s="13">
+        <v>0</v>
+      </c>
+      <c r="M17" s="14">
+        <v>45798</v>
+      </c>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
       <c r="P17" s="13"/>
@@ -2157,26 +2201,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65613A53-C102-4256-AEC9-305787A9B0EA}">
   <dimension ref="A1:P6"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.875" style="1"/>
-    <col min="2" max="2" width="8.875" style="2"/>
-    <col min="3" max="3" width="8.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="8.83203125" style="2"/>
+    <col min="3" max="3" width="8.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.58203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.58203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.08203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.25" style="1" customWidth="1"/>
-    <col min="11" max="12" width="10.625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="17.125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="10.58203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.08203125" style="1" customWidth="1"/>
     <col min="14" max="15" width="17" style="1" customWidth="1"/>
     <col min="16" max="16" width="38.5" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.875" style="1"/>
+    <col min="17" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30">
+    <row r="1" spans="1:16" ht="28">
       <c r="A1" s="21"/>
       <c r="B1" s="19" t="s">
         <v>0</v>
@@ -2232,7 +2276,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D2" s="20"/>
       <c r="E2" s="21">
@@ -2407,26 +2451,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF0F1BD-DA81-409F-B879-31CA2FD3E4BB}">
   <dimension ref="A1:P6"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.875" style="1"/>
-    <col min="2" max="2" width="8.875" style="2"/>
-    <col min="3" max="3" width="8.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="8.83203125" style="2"/>
+    <col min="3" max="3" width="8.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.58203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.58203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.08203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.25" style="1" customWidth="1"/>
-    <col min="11" max="12" width="10.625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="17.125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="10.58203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.08203125" style="1" customWidth="1"/>
     <col min="14" max="15" width="17" style="1" customWidth="1"/>
     <col min="16" max="16" width="38.5" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.875" style="1"/>
+    <col min="17" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30">
+    <row r="1" spans="1:16" ht="28">
       <c r="A1" s="26"/>
       <c r="B1" s="24" t="s">
         <v>0</v>
@@ -2482,7 +2526,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D2" s="25"/>
       <c r="E2" s="26">
@@ -2655,13 +2699,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22554d0a-1932-447e-b007-a2186b2152bd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2849,26 +2892,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22554d0a-1932-447e-b007-a2186b2152bd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D844D4EE-45BA-4D0C-B92D-0FE188981EFA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D86BB587-35FF-4C72-A3B4-30D223CD8217}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="22554d0a-1932-447e-b007-a2186b2152bd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2892,9 +2928,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D86BB587-35FF-4C72-A3B4-30D223CD8217}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D844D4EE-45BA-4D0C-B92D-0FE188981EFA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="22554d0a-1932-447e-b007-a2186b2152bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Atualiza planilha via painel SAVAL (10/07/2026, 14:15:51)
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q19"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="str">
@@ -448,6 +448,9 @@
       <c r="P1" t="str">
         <v>OBS. LUCIANA</v>
       </c>
+      <c r="Q1" t="str">
+        <v>ANDAMENTO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -489,6 +492,9 @@
       <c r="M2" t="str">
         <v>05/28/2026</v>
       </c>
+      <c r="Q2" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
@@ -527,6 +533,9 @@
       <c r="M3" t="str">
         <v>05/27/2026</v>
       </c>
+      <c r="Q3" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="str">
@@ -565,6 +574,9 @@
       <c r="M4" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q4" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="str">
@@ -603,6 +615,9 @@
       <c r="M5" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q5" t="str">
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
@@ -641,6 +656,9 @@
       <c r="M6" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q6" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
@@ -679,6 +697,9 @@
       <c r="M7" t="str">
         <v>07/01/2026</v>
       </c>
+      <c r="Q7" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
@@ -717,6 +738,9 @@
       <c r="M8" t="str">
         <v>05/22/2026</v>
       </c>
+      <c r="Q8" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="str">
@@ -755,6 +779,9 @@
       <c r="M9" t="str">
         <v>05/22/2026</v>
       </c>
+      <c r="Q9" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="str">
@@ -793,6 +820,9 @@
       <c r="M10" t="str">
         <v>05/22/2026</v>
       </c>
+      <c r="Q10" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="str">
@@ -831,6 +861,9 @@
       <c r="M11" t="str">
         <v>05/22/2026</v>
       </c>
+      <c r="Q11" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="str">
@@ -869,6 +902,9 @@
       <c r="M12" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q12" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="str">
@@ -907,6 +943,9 @@
       <c r="M13" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q13" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" t="str">
@@ -945,6 +984,9 @@
       <c r="M14" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q14" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" t="str">
@@ -968,6 +1010,9 @@
       <c r="H15">
         <v>0</v>
       </c>
+      <c r="Q15" t="str">
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" t="str">
@@ -991,6 +1036,21 @@
       <c r="H16">
         <v>0</v>
       </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" t="str">
@@ -1029,6 +1089,9 @@
       <c r="M17" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q17" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="18">
       <c r="B18" t="str">
@@ -1052,6 +1115,21 @@
       <c r="H18">
         <v>2</v>
       </c>
+      <c r="I18">
+        <v>5</v>
+      </c>
+      <c r="J18">
+        <v>5</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" t="str">
@@ -1071,6 +1149,9 @@
       </c>
       <c r="H19">
         <v>0</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Pendente</v>
       </c>
     </row>
   </sheetData>
@@ -1079,14 +1160,14 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="str">
@@ -1134,6 +1215,9 @@
       <c r="P1" t="str">
         <v>OBS. LUCIANA</v>
       </c>
+      <c r="Q1" t="str">
+        <v>ANDAMENTO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1175,6 +1259,9 @@
       <c r="M2" t="str">
         <v>05/28/2026</v>
       </c>
+      <c r="Q2" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
@@ -1213,6 +1300,9 @@
       <c r="M3" t="str">
         <v>05/28/2026</v>
       </c>
+      <c r="Q3" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="str">
@@ -1251,6 +1341,9 @@
       <c r="M4" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q4" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="str">
@@ -1289,6 +1382,9 @@
       <c r="M5" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q5" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
@@ -1327,6 +1423,9 @@
       <c r="M6" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q6" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
@@ -1365,6 +1464,9 @@
       <c r="M7" t="str">
         <v>07/01/2026</v>
       </c>
+      <c r="Q7" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
@@ -1403,6 +1505,9 @@
       <c r="M8" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q8" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="str">
@@ -1441,6 +1546,9 @@
       <c r="M9" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q9" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="str">
@@ -1479,6 +1587,9 @@
       <c r="M10" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q10" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="str">
@@ -1517,6 +1628,9 @@
       <c r="M11" t="str">
         <v>05/22/2026</v>
       </c>
+      <c r="Q11" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="str">
@@ -1555,6 +1669,9 @@
       <c r="M12" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q12" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="str">
@@ -1593,6 +1710,9 @@
       <c r="M13" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q13" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" t="str">
@@ -1616,6 +1736,9 @@
       <c r="H14">
         <v>0</v>
       </c>
+      <c r="Q14" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" t="str">
@@ -1639,6 +1762,9 @@
       <c r="H15">
         <v>0</v>
       </c>
+      <c r="Q15" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" t="str">
@@ -1662,6 +1788,9 @@
       <c r="H16">
         <v>0</v>
       </c>
+      <c r="Q16" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" t="str">
@@ -1700,6 +1829,9 @@
       <c r="M17" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q17" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="18">
       <c r="B18" t="str">
@@ -1738,6 +1870,9 @@
       <c r="M18" t="str">
         <v>05/21/2026</v>
       </c>
+      <c r="Q18" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" t="str">
@@ -1758,6 +1893,9 @@
       <c r="H19">
         <v>0</v>
       </c>
+      <c r="Q19" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" t="str">
@@ -1778,6 +1916,9 @@
       <c r="H20">
         <v>0</v>
       </c>
+      <c r="Q20" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="21">
       <c r="B21" t="str">
@@ -1797,6 +1938,9 @@
       </c>
       <c r="H21">
         <v>0</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Pendente</v>
       </c>
     </row>
   </sheetData>
@@ -1805,7 +1949,7 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1860,6 +2004,9 @@
       <c r="P1" t="str">
         <v>OBS. LUCIANA</v>
       </c>
+      <c r="Q1" t="str">
+        <v>ANDAMENTO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1883,6 +2030,9 @@
       <c r="H2">
         <v>15</v>
       </c>
+      <c r="Q2" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
@@ -1918,6 +2068,9 @@
       <c r="M3" t="str">
         <v>07/01/2026</v>
       </c>
+      <c r="Q3" t="str">
+        <v>Pendente</v>
+      </c>
       <c r="R3" t="str">
         <v>TURMA A</v>
       </c>
@@ -1956,6 +2109,9 @@
       <c r="M4" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q4" t="str">
+        <v>Pendente</v>
+      </c>
       <c r="S4" t="str">
         <v>DAMAZ</v>
       </c>
@@ -1979,6 +2135,9 @@
       <c r="H5">
         <v>23</v>
       </c>
+      <c r="Q5" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
@@ -1998,6 +2157,9 @@
       </c>
       <c r="H6">
         <v>0</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Pendente</v>
       </c>
     </row>
   </sheetData>
@@ -2013,7 +2175,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:Q12"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="str">
@@ -2061,6 +2223,9 @@
       <c r="P1" t="str">
         <v>OBS. LUCIANA</v>
       </c>
+      <c r="Q1" t="str">
+        <v>ANDAMENTO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2084,6 +2249,9 @@
       <c r="H2">
         <v>15</v>
       </c>
+      <c r="Q2" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
@@ -2119,6 +2287,9 @@
       <c r="M3" t="str">
         <v>07/01/2026</v>
       </c>
+      <c r="Q3" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="str">
@@ -2154,6 +2325,9 @@
       <c r="M4" t="str">
         <v>05/21/2025</v>
       </c>
+      <c r="Q4" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="str">
@@ -2174,6 +2348,9 @@
       <c r="H5">
         <v>23</v>
       </c>
+      <c r="Q5" t="str">
+        <v>Pendente</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
@@ -2194,8 +2371,8 @@
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="L6">
-        <v>1</v>
+      <c r="Q6" t="str">
+        <v>Pendente</v>
       </c>
     </row>
     <row r="12">
@@ -2209,7 +2386,7 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza planilha via painel SAVAL (10/07/2026, 15:34:30)
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -616,7 +616,7 @@
         <v>05/21/2026</v>
       </c>
       <c r="Q5" t="str">
-        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
+        <v>Pendente</v>
       </c>
     </row>
     <row r="6">
@@ -1042,14 +1042,8 @@
       <c r="J16">
         <v>3</v>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
       <c r="Q16" t="str">
-        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
+        <v>Pendente</v>
       </c>
     </row>
     <row r="17">
@@ -1121,12 +1115,6 @@
       <c r="J18">
         <v>5</v>
       </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
       <c r="Q18" t="str">
         <v>Pendente</v>
       </c>
@@ -1151,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
   </sheetData>
@@ -1736,6 +1724,15 @@
       <c r="H14">
         <v>0</v>
       </c>
+      <c r="I14">
+        <v>6</v>
+      </c>
+      <c r="J14">
+        <v>17</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
       <c r="Q14" t="str">
         <v>Pendente</v>
       </c>
@@ -1762,6 +1759,12 @@
       <c r="H15">
         <v>0</v>
       </c>
+      <c r="I15">
+        <v>8</v>
+      </c>
+      <c r="J15">
+        <v>2</v>
+      </c>
       <c r="Q15" t="str">
         <v>Pendente</v>
       </c>
@@ -1788,6 +1791,12 @@
       <c r="H16">
         <v>0</v>
       </c>
+      <c r="I16">
+        <v>8</v>
+      </c>
+      <c r="J16">
+        <v>2</v>
+      </c>
       <c r="Q16" t="str">
         <v>Pendente</v>
       </c>
@@ -1893,6 +1902,12 @@
       <c r="H19">
         <v>0</v>
       </c>
+      <c r="I19">
+        <v>8</v>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
       <c r="Q19" t="str">
         <v>Pendente</v>
       </c>
@@ -1916,6 +1931,9 @@
       <c r="H20">
         <v>0</v>
       </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
       <c r="Q20" t="str">
         <v>Pendente</v>
       </c>
@@ -1940,7 +1958,7 @@
         <v>0</v>
       </c>
       <c r="Q21" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
   </sheetData>
@@ -2135,6 +2153,15 @@
       <c r="H5">
         <v>23</v>
       </c>
+      <c r="I5">
+        <v>8</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>15</v>
+      </c>
       <c r="Q5" t="str">
         <v>Pendente</v>
       </c>
@@ -2156,6 +2183,9 @@
         <v>0</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
       <c r="Q6" t="str">
@@ -2249,6 +2279,12 @@
       <c r="H2">
         <v>15</v>
       </c>
+      <c r="I2">
+        <v>7</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
       <c r="Q2" t="str">
         <v>Pendente</v>
       </c>
@@ -2349,7 +2385,7 @@
         <v>23</v>
       </c>
       <c r="Q5" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="6">
@@ -2372,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Atualiza planilha via painel SAVAL (13/07/2026, 09:46:45)
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -1734,7 +1734,7 @@
         <v>4</v>
       </c>
       <c r="Q14" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="15">
@@ -1766,7 +1766,7 @@
         <v>2</v>
       </c>
       <c r="Q15" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="16">
@@ -1798,7 +1798,7 @@
         <v>2</v>
       </c>
       <c r="Q16" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="17">
@@ -1909,7 +1909,7 @@
         <v>2</v>
       </c>
       <c r="Q19" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="20">
@@ -1935,7 +1935,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="21">
@@ -2163,7 +2163,7 @@
         <v>15</v>
       </c>
       <c r="Q5" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="6">
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha via painel SAVAL (13/07/2026, 10:05:42)
</commit_message>
<xml_diff>
--- a/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
+++ b/CONTROLE RECURSOS HUMANOS - PLANO DE AULA.xlsx
@@ -1043,7 +1043,7 @@
         <v>3</v>
       </c>
       <c r="Q16" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="17">
@@ -1116,7 +1116,7 @@
         <v>5</v>
       </c>
       <c r="Q18" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="19">
@@ -2048,8 +2048,14 @@
       <c r="H2">
         <v>15</v>
       </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <v>8</v>
+      </c>
       <c r="Q2" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="3">
@@ -2286,7 +2292,7 @@
         <v>1</v>
       </c>
       <c r="Q2" t="str">
-        <v>Pendente</v>
+        <v>PendenteRevisado para envioEnviadoSem plano de aula</v>
       </c>
     </row>
     <row r="3">

</xml_diff>